<commit_message>
Account for the rejected programmes, not only the viable ones
The workbook listed the 81 programmes that passed the filters but only
22 of the many the research checked and ruled out, so it recorded what
to apply to without recording what had already been eliminated or why.

The Excluded sheet now carries 83 entries with the reason and a
category: German programmes whose published grade bars he misses (his
converted grade is 3.0-3.4), French programmes that admit at M1 with
zero tuition but require an apprenticeship contract obtainable only
after a visa, Italian Master di I livello and Spanish titulos propios
that are not second-cycle degrees, private schools failing
accreditation including one rated H- by anabin, and the Erasmus Mundus
data programmes that all require a computing first degree.

All three main sheets now carry autofilters.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0143Vz9N8sock2hiEbrM34ZT
</commit_message>
<xml_diff>
--- a/output/masters-research.xlsx
+++ b/output/masters-research.xlsx
@@ -16,6 +16,10 @@
     <sheet name="Action plan" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="Excluded" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
+  <definedNames>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'All programmes'!$A$4:$J$85</definedName>
+    <definedName function="false" hidden="true" localSheetId="6" name="_xlnm._FilterDatabase" vbProcedure="false">Excluded!$A$4:$D$87</definedName>
+  </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -26,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1553" uniqueCount="770">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1848" uniqueCount="922">
   <si>
     <t xml:space="preserve">European Master's Research — Results</t>
   </si>
@@ -2212,31 +2216,463 @@
     <t xml:space="preserve">Missing either costs real money</t>
   </si>
   <si>
-    <t xml:space="preserve">Checked and excluded — so you do not rediscover them</t>
-  </si>
-  <si>
-    <t xml:space="preserve">What</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Why excluded</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Every Italian "music business master" — LUISS BS, Sapienza MMCM, Roma Tre, IULM, 24ORE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All Master di I livello: 1 year, 60-65 CFU. Not a second-cycle degree</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nearly every Spanish "master en industria musical" — UC3M, IL3-UB, UAM, SAE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Formacion permanente / titulo propio. Likely fails the EQF-6 test for Spain's post-study permit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Every French Mastere Specialise, without exception</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CGE rules require Bac+5 (or Bac+4 + 3 years). He holds Bac+3. Not a diplome national; confers no grade de master</t>
+    <t xml:space="preserve">Checked and rejected - so you do not rediscover them</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every programme or institution the research examined and ruled out, with the reason. This is the other half of the picture: 81 passed the filters, these did not.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Institution / programme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Why it was rejected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TH Nurnberg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minimum grade 1.5, plus GMAT 550 for 1.5-2.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grade bar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hochschule Pforzheim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minimum grade 2.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">THM / Hochschule Mittelhessen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minimum 2.3, plus 210 ECTS and German B1 - three walls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FH Munster</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minimum grade 2.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hochschule Bremen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hochschule Hof</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minimum grade 2.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HNU Neu-Ulm (4 programmes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TH Koln</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hochschule Mainz (2 programmes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hochschule Rhine-Waal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OVGU Magdeburg IMME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minimum 2.9 - the most generous in Germany, and he still misses it</t>
+  </si>
+  <si>
+    <t xml:space="preserve">htw saar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minimum grade 2.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hochschule Bonn-Rhein-Sieg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vergabeverordnung NRW: only 2 places for non-EU, needing CGPA ~1.0-1.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non-EU quota</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCI Innsbruck</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EUR 8,250/semester = EUR 16,500/yr - fails the cost filter outright</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IMC Krems</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EUR 6,900/sem, and prints "minimum 180 ECTS lasting at least six semesters" verbatim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost + 180 rule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FH Technikum Wien</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EUR 3,000/semester</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FH Wiener Neustadt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EUR 850/semester, and demands a certificate not an MOI letter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WU Wien</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requires "at least 180 ECTS with 45 ECTS in business administration"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">180 rule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Universitat Wien</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accepts MOI letters only from EU/EEA/CH/UK/US/AU/NZ/CA institutions - structurally excludes Tunisia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IAE Lille - SMRC / MBX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free and M1-entry, but requires a signed French apprenticeship contract before enrolment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alternance trap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IAE Caen - Digital &amp; Social Media</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alternance-mandatory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paris-Saclay - MRC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISM-IAE Versailles - MRC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Exclusivement en alternance", 24-month contract from M1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IAE Montpellier - CSRC (Microsoft, pure CRM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perfect CRM fit but alternance-mandatory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IAE Bretagne Sud - Marketing digital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Digitalisation de la relation-client" but alternance-mandatory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IAE Angers - digital M2s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M1 is fine but both digital M2 exits are alternance-only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IAE Orleans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alternance-only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IAE Brest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IAE Limoges</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No marketing master at all</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nothing suitable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IAE Pau-Bayonne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">International trade only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IAE Perpignan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2-only entry - he has no M1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2-only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IAE Rouen / Toulon / Paris Cite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Excluded on entry route</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2-only / alternance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IAE Valenciennes - MDC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ambiguous format; institution gave an email address instead of a published rule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IAE Savoie - Marketing Cursus International</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FI with a CRM module, but hard-gated on a TOEIC/IELTS certificate he does not have</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every French Mastere Specialise</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CGE rules require Bac+5 (or Bac+4 + 3 years). He holds Bac+3. Not a diplome national</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Degree level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESART (advertises a "Mastere Specialise")</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not a CGE member; RNCP registration expiring 31 Aug 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accreditation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Queen's University Belfast</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GBP 23,000/yr for international students, against GBP 7,700 for locals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ulster University</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GBP 18,310/yr international</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UK music-business masters generally</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GBP 16,000-31,900. Only Westminster survives as a stretch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UGent - Marketing Analysis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">An ADVANCED master requiring a bachelor AND a master, or a 4-year bachelor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hautes ecoles (HELMo, HEPL, HE Vinci, HEH)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Offer marketing only at bachelor level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flemish hogescholen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Award no business masters at all since the 2013 integratie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">THUAS The Hague</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EUR 19,700 - fails cost and one other filter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saxion MBA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Part-time - carries NO student visa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No visa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HvA Applied AI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dutch-taught only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All Dutch WO masters (if Licence Fondamentale)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nuffic rates Fondamentale as 2 years of WO - below a Dutch bachelor. Pre-masters capped at 60 EC cannot bridge a full year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Utrecht pre-master</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bars students who need a residence permit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LUISS Business School - music</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Master di I livello: 1 year, 60-65 CFU. Not a second-cycle degree</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sapienza MMCM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Master di I livello</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roma Tre / IULM / 24ORE music masters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saint Louis College of Music, Rome</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Genuinely AFAM-accredited, but its music-business master is still I livello</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Milano Statale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~EUR 3,394/yr - Tunisia is Group C and ISEE parificato is EXPLICITLY FORBIDDEN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coimbra Business School music-industries course</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A pos-graduacao, not a master</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UC3M music industry master</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Titulo propio / formacion permanente - EUR 5,900. Likely fails EQF-6 for the post-study permit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IL3-UB / UAM / SAE music masters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Titulo propio - not state masters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UC3M Madrid - English marketing master</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EUR 13,500 and C1 English required - stretch on both counts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost + English</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uniarts Helsinki - MA Music Business</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perfect subject fit; EUR 28,000/yr with a VERIFIED zero-scholarship position</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Swedish universities generally</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EUR 9,000-17,100/yr, and Tunisia is not among the Swedish Institute 34 eligible countries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost + funding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">University of Skovde (best Swedish waiver)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50% waiver sits on a games/informatics faculty - matches none of his directions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mismatch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finnish universities of applied sciences</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Require 2 years of relevant work experience - he has an internship</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experience</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oslo and Bergen universities</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EUR 16,000-32,000/yr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BI Norwegian Business School</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EUR 13,650/yr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rome Business School</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Awards a Spanish VIU titulo propio, not an Italian degree</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EU Business School</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Germany/Spain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rated H- by Germany anabin. Degrees from Roehampton/Derby/UCAM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSBI Berlin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Awards no German degree</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IMB Barcelona</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EUNEIZ titulo propio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISEG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNCP titles valid but no grade, no visa, not CGE, no AACSB/EQUIS/AMBA, and bac+5 tracks are alternance-only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESSCA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requires a 4-year bachelor OR 3 years experience - he has neither</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entry</t>
   </si>
   <si>
     <t xml:space="preserve">Berklee Valencia</t>
@@ -2245,97 +2681,121 @@
     <t xml:space="preserve">~EUR 48,000</t>
   </si>
   <si>
-    <t xml:space="preserve">Uniarts Helsinki MA Music Business</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Perfect subject fit, EUR 28,000/yr, verified zero scholarships</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UK music-business master's generally</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GBP 16,000-31,900. Only Westminster survives as a stretch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Popakademie, BIMM, Catalyst Berlin, SAE, ICMP, Saint Louis Rome</t>
+    <t xml:space="preserve">Popakademie, BIMM, Catalyst Berlin, SAE, ICMP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Various</t>
   </si>
   <si>
     <t xml:space="preserve">Fail on accreditation, price, or both</t>
   </si>
   <si>
-    <t xml:space="preserve">Rome Business School</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Awards a Spanish titulo propio, not an Italian degree</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EU Business School</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rated H- by Germany's anabin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BSBI Berlin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Awards no German degree</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IMB Barcelona</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EUNEIZ titulo propio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ISEG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RNCP titles valid but no grade, no visa, not CGE, no AACSB/EQUIS/AMBA, and bac+5 tracks are alternance-only</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ESSCA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Requires a 4-year bachelor or 3 years' experience</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All AI/data Erasmus Mundus programmes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Every one requires a CS, engineering or maths first degree</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMMIE (Erasmus Mundus)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Requires 240 ECTS — unrecoverable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Queen's Belfast (GBP 23,000) and Ulster (GBP 18,310)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Northern Ireland is not the cheap UK route it appears to be</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finnish universities of applied sciences</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Require 2 years' relevant work experience</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Explicit "at least 3 years, at least 180 ECTS", applied strictly</t>
+    <t xml:space="preserve">Accreditation + cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All AI/data Erasmus Mundus (BDMA, EMAI, DEAI, EDISS, CoDaS, NeuroData, MULTICOM, EMLDS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every one requires a CS, engineering or maths first degree - hard blocks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMMIE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requires 240 ECTS - unrecoverable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Credits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KTU marketing and big-data masters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lithuanian-taught only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MRU Communication and Digital Marketing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is a BACHELOR, not a master</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Turiba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latvia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only an EUR 3,550 MBA; official page bot-blocked</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUBG / UNWE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bulgaria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Out of range / publishes no English master fee at all</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost / NOT VERIFIED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUEB and Greek masters generally</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Require a C2 English diploma, and DOATAP recognition is where 146 gets challenged with no safety valve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">English + credits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">University of Luxembourg - Entrepreneurship &amp; Innovation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">States "BA degree with 180 ECTS" three times with NO complementary-credit fallback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">University of Luxembourg - Data Science</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EUR 800/yr but demands linear algebra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prerequisite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">University of Silesia - Creative Management in New Media</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requires an arts/media bachelor PLUS a portfolio review</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portfolio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cyprus generally</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Labour market test - jobs go to Cypriots and EU citizens first</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Job market</t>
   </si>
   <si>
     <t xml:space="preserve">German Studienkolleg</t>
   </si>
   <si>
-    <t xml:space="preserve">Bachelor entry only — irrelevant to master's applicants</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IAE Lille, IAE Caen, Paris-Saclay (free M1 routes)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Require a signed French apprenticeship contract before enrolment — unobtainable pre-visa</t>
+    <t xml:space="preserve">Bachelor entry only - irrelevant to master applicants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not applicable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Swiss universities</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Explicit "at least 3 years, at least 180 ECTS", applied strictly; HES-SO adds work experience</t>
   </si>
 </sst>
 </file>
@@ -2560,6 +3020,39 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="4">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF1F4E79"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2F2F2"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -2621,6 +3114,14 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7394,6 +7895,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A4:J85"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -7401,6 +7903,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -8797,11 +9300,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:D87"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="80"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8809,19 +9314,22 @@
         <v>728</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="s">
         <v>729</v>
       </c>
-      <c r="B3" s="5" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
         <v>730</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+      <c r="B4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>731</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="D4" s="5" t="s">
         <v>732</v>
       </c>
     </row>
@@ -8830,39 +9338,69 @@
         <v>733</v>
       </c>
       <c r="B5" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>734</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>735</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
+        <v>736</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>737</v>
+      </c>
+      <c r="D6" s="6" t="s">
         <v>735</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>736</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>738</v>
+        <v>53</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>739</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>735</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>740</v>
+        <v>53</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>741</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>735</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
+        <v>742</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9" s="6" t="s">
         <v>741</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>742</v>
+      <c r="D9" s="6" t="s">
+        <v>735</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8870,7 +9408,13 @@
         <v>743</v>
       </c>
       <c r="B10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C10" s="6" t="s">
         <v>744</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>735</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8878,87 +9422,153 @@
         <v>745</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>746</v>
+        <v>53</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>744</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>735</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>748</v>
+        <v>53</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>744</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>735</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>750</v>
+        <v>53</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>744</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>735</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>751</v>
+        <v>748</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>752</v>
+        <v>53</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>744</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>735</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>753</v>
+        <v>749</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>754</v>
+        <v>53</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>750</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>735</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>756</v>
+        <v>53</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>752</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>735</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>757</v>
+        <v>753</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>758</v>
+        <v>53</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>754</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>755</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>759</v>
+        <v>756</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>760</v>
+        <v>71</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>757</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>758</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
+        <v>759</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>760</v>
+      </c>
+      <c r="D19" s="6" t="s">
         <v>761</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>762</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
+        <v>762</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C20" s="6" t="s">
         <v>763</v>
       </c>
-      <c r="B20" s="6" t="s">
-        <v>764</v>
+      <c r="D20" s="6" t="s">
+        <v>758</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>578</v>
+        <v>764</v>
       </c>
       <c r="B21" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C21" s="6" t="s">
         <v>765</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>758</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8966,18 +9576,927 @@
         <v>766</v>
       </c>
       <c r="B22" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C22" s="6" t="s">
         <v>767</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>768</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
+        <v>769</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>770</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="7" t="s">
+        <v>771</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>772</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="7" t="s">
+        <v>774</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>775</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="7" t="s">
+        <v>776</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>775</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="7" t="s">
+        <v>777</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>778</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="7" t="s">
+        <v>779</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>780</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="7" t="s">
+        <v>781</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>782</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="7" t="s">
+        <v>783</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>784</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="7" t="s">
+        <v>785</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>786</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="7" t="s">
+        <v>787</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>786</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="7" t="s">
+        <v>788</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>789</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="7" t="s">
+        <v>791</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>792</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="7" t="s">
+        <v>793</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>794</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="7" t="s">
+        <v>796</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>797</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="7" t="s">
+        <v>799</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>800</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="7" t="s">
+        <v>801</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>802</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="7" t="s">
+        <v>803</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>804</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="7" t="s">
+        <v>806</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>807</v>
+      </c>
+      <c r="D40" s="6" t="s">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="7" t="s">
+        <v>809</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>388</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>810</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="7" t="s">
+        <v>811</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>388</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>812</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="7" t="s">
+        <v>813</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>388</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>814</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="7" t="s">
+        <v>815</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>816</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="7" t="s">
+        <v>817</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>818</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="7" t="s">
+        <v>819</v>
+      </c>
+      <c r="B46" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>820</v>
+      </c>
+      <c r="D46" s="6" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="7" t="s">
+        <v>821</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>822</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="7" t="s">
+        <v>823</v>
+      </c>
+      <c r="B48" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>824</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="7" t="s">
+        <v>826</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>827</v>
+      </c>
+      <c r="D49" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="7" t="s">
+        <v>828</v>
+      </c>
+      <c r="B50" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>829</v>
+      </c>
+      <c r="D50" s="6" t="s">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="7" t="s">
+        <v>831</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>832</v>
+      </c>
+      <c r="D51" s="6" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="7" t="s">
+        <v>833</v>
+      </c>
+      <c r="B52" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C52" s="6" t="s">
+        <v>834</v>
+      </c>
+      <c r="D52" s="6" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="7" t="s">
+        <v>835</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>836</v>
+      </c>
+      <c r="D53" s="6" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="7" t="s">
+        <v>837</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>836</v>
+      </c>
+      <c r="D54" s="6" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="7" t="s">
+        <v>838</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>839</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="7" t="s">
+        <v>840</v>
+      </c>
+      <c r="B56" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>841</v>
+      </c>
+      <c r="D56" s="6" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="7" t="s">
+        <v>842</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>843</v>
+      </c>
+      <c r="D57" s="6" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="7" t="s">
+        <v>844</v>
+      </c>
+      <c r="B58" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="C58" s="6" t="s">
+        <v>845</v>
+      </c>
+      <c r="D58" s="6" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="7" t="s">
+        <v>846</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>847</v>
+      </c>
+      <c r="D59" s="6" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="7" t="s">
+        <v>848</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>849</v>
+      </c>
+      <c r="D60" s="6" t="s">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="7" t="s">
+        <v>851</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>852</v>
+      </c>
+      <c r="D61" s="6" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="7" t="s">
+        <v>853</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>562</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>854</v>
+      </c>
+      <c r="D62" s="6" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="7" t="s">
+        <v>856</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>562</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>857</v>
+      </c>
+      <c r="D63" s="6" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="7" t="s">
+        <v>859</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>860</v>
+      </c>
+      <c r="D64" s="6" t="s">
+        <v>861</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="7" t="s">
+        <v>862</v>
+      </c>
+      <c r="B65" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>863</v>
+      </c>
+      <c r="D65" s="6" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="7" t="s">
+        <v>864</v>
+      </c>
+      <c r="B66" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>865</v>
+      </c>
+      <c r="D66" s="6" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="7" t="s">
+        <v>866</v>
+      </c>
+      <c r="B67" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>867</v>
+      </c>
+      <c r="D67" s="6" t="s">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="7" t="s">
+        <v>868</v>
+      </c>
+      <c r="B68" s="6" t="s">
+        <v>869</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>870</v>
+      </c>
+      <c r="D68" s="6" t="s">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="7" t="s">
+        <v>871</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C69" s="6" t="s">
+        <v>872</v>
+      </c>
+      <c r="D69" s="6" t="s">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="7" t="s">
+        <v>873</v>
+      </c>
+      <c r="B70" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="C70" s="6" t="s">
+        <v>874</v>
+      </c>
+      <c r="D70" s="6" t="s">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="7" t="s">
+        <v>875</v>
+      </c>
+      <c r="B71" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>876</v>
+      </c>
+      <c r="D71" s="6" t="s">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="7" t="s">
+        <v>878</v>
+      </c>
+      <c r="B72" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C72" s="6" t="s">
+        <v>879</v>
+      </c>
+      <c r="D72" s="6" t="s">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="7" t="s">
+        <v>881</v>
+      </c>
+      <c r="B73" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>882</v>
+      </c>
+      <c r="D73" s="6" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="7" t="s">
+        <v>883</v>
+      </c>
+      <c r="B74" s="6" t="s">
+        <v>884</v>
+      </c>
+      <c r="C74" s="6" t="s">
+        <v>885</v>
+      </c>
+      <c r="D74" s="6" t="s">
+        <v>886</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="7" t="s">
+        <v>887</v>
+      </c>
+      <c r="B75" s="6" t="s">
+        <v>603</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>888</v>
+      </c>
+      <c r="D75" s="6" t="s">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="7" t="s">
+        <v>889</v>
+      </c>
+      <c r="B76" s="6" t="s">
+        <v>603</v>
+      </c>
+      <c r="C76" s="6" t="s">
+        <v>890</v>
+      </c>
+      <c r="D76" s="6" t="s">
+        <v>891</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="7" t="s">
+        <v>892</v>
+      </c>
+      <c r="B77" s="6" t="s">
+        <v>394</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>893</v>
+      </c>
+      <c r="D77" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="7" t="s">
+        <v>894</v>
+      </c>
+      <c r="B78" s="6" t="s">
+        <v>394</v>
+      </c>
+      <c r="C78" s="6" t="s">
+        <v>895</v>
+      </c>
+      <c r="D78" s="6" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="7" t="s">
+        <v>896</v>
+      </c>
+      <c r="B79" s="6" t="s">
+        <v>897</v>
+      </c>
+      <c r="C79" s="6" t="s">
+        <v>898</v>
+      </c>
+      <c r="D79" s="6" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="7" t="s">
+        <v>899</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>900</v>
+      </c>
+      <c r="C80" s="6" t="s">
+        <v>901</v>
+      </c>
+      <c r="D80" s="6" t="s">
+        <v>902</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="7" t="s">
+        <v>903</v>
+      </c>
+      <c r="B81" s="6" t="s">
+        <v>568</v>
+      </c>
+      <c r="C81" s="6" t="s">
+        <v>904</v>
+      </c>
+      <c r="D81" s="6" t="s">
+        <v>905</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="7" t="s">
+        <v>906</v>
+      </c>
+      <c r="B82" s="6" t="s">
+        <v>573</v>
+      </c>
+      <c r="C82" s="6" t="s">
+        <v>907</v>
+      </c>
+      <c r="D82" s="6" t="s">
         <v>768</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>769</v>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="7" t="s">
+        <v>908</v>
+      </c>
+      <c r="B83" s="6" t="s">
+        <v>573</v>
+      </c>
+      <c r="C83" s="6" t="s">
+        <v>909</v>
+      </c>
+      <c r="D83" s="6" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="7" t="s">
+        <v>911</v>
+      </c>
+      <c r="B84" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C84" s="6" t="s">
+        <v>912</v>
+      </c>
+      <c r="D84" s="6" t="s">
+        <v>913</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="7" t="s">
+        <v>914</v>
+      </c>
+      <c r="B85" s="6" t="s">
+        <v>384</v>
+      </c>
+      <c r="C85" s="6" t="s">
+        <v>915</v>
+      </c>
+      <c r="D85" s="6" t="s">
+        <v>916</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="7" t="s">
+        <v>917</v>
+      </c>
+      <c r="B86" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C86" s="6" t="s">
+        <v>918</v>
+      </c>
+      <c r="D86" s="6" t="s">
+        <v>919</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="7" t="s">
+        <v>920</v>
+      </c>
+      <c r="B87" s="6" t="s">
+        <v>578</v>
+      </c>
+      <c r="C87" s="6" t="s">
+        <v>921</v>
+      </c>
+      <c r="D87" s="6" t="s">
+        <v>768</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A4:D87"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -8985,5 +10504,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>